<commit_message>
add ADM-CAT-FUN-003 ADM-CAT-FUN-004 ADM-CAT-FUN-005 ADM-CAT-FUN-006 ADM-CAT-FUN-007 ADM-CAT-FUN-008 ADM-CAT-FUN-009 ADM-CAT-VAL-002 ADM-CAT-VAL-003 ADM-CAT-VAL-004
</commit_message>
<xml_diff>
--- a/deepshika.xlsx
+++ b/deepshika.xlsx
@@ -997,7 +997,7 @@
 2. Slug field displays an appropriate required-field validation message.</v>
       </c>
       <c r="N16" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R16" t="str">
         <v>Staging</v>
@@ -1057,7 +1057,7 @@
 2. Appropriate validation is displayed for both required fields.</v>
       </c>
       <c r="N17" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R17" t="str">
         <v>Staging</v>
@@ -1120,7 +1120,7 @@
 3. Created category displays the selected parent correctly.</v>
       </c>
       <c r="N18" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R18" t="str">
         <v>Staging</v>
@@ -1181,7 +1181,7 @@
 2. Category A (10) appears before Category B (20), following the rule that lower numbers appear first.</v>
       </c>
       <c r="N19" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R19" t="str">
         <v>Staging</v>
@@ -1240,7 +1240,7 @@
 3. Uploaded icon is associated with the category.</v>
       </c>
       <c r="N20" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R20" t="str">
         <v>Staging</v>
@@ -1298,7 +1298,7 @@
         <v>System should reject the invalid slug or normalize it according to the application's defined slug rules. Category should not be created with an invalid slug.</v>
       </c>
       <c r="N21" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R21" t="str">
         <v>Staging</v>
@@ -1359,7 +1359,7 @@
 3. Category is not visible on the public website if Active controls website visibility.</v>
       </c>
       <c r="N22" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R22" t="str">
         <v>Staging</v>
@@ -1417,7 +1417,7 @@
 3. Existing category list remains unchanged.</v>
       </c>
       <c r="N23" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R23" t="str">
         <v>Staging</v>
@@ -1482,7 +1482,7 @@
 4. Updated values are displayed correctly in the category list.</v>
       </c>
       <c r="N24" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R24" t="str">
         <v>Staging</v>

</xml_diff>

<commit_message>
add ADM-CAT-FUN-010 ADM-CAT-FUN-011 ADM-CAT-FUN-012 ADM-CAT-FUN-013 ADM-CAT-NEG-001
</commit_message>
<xml_diff>
--- a/deepshika.xlsx
+++ b/deepshika.xlsx
@@ -1603,7 +1603,7 @@
 3. Category is no longer visible on the public website if Hide controls website visibility.</v>
       </c>
       <c r="N26" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R26" t="str">
         <v>Staging</v>
@@ -1662,7 +1662,7 @@
 3. No unintended changes are made.</v>
       </c>
       <c r="N27" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R27" t="str">
         <v>Staging</v>
@@ -1723,7 +1723,7 @@
 3. Deleted category no longer appears in the category list/search results.</v>
       </c>
       <c r="N28" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R28" t="str">
         <v>Staging</v>
@@ -1781,7 +1781,7 @@
 2. Category remains unchanged and available in the category list.</v>
       </c>
       <c r="N29" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R29" t="str">
         <v>Staging</v>
@@ -1839,7 +1839,7 @@
         <v>System should prevent unsafe deletion or handle the in-use dependency according to the defined business rule, with a clear message where applicable.</v>
       </c>
       <c r="N30" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R30" t="str">
         <v>Staging</v>

</xml_diff>

<commit_message>
update step 3 wizard
</commit_message>
<xml_diff>
--- a/deepshika.xlsx
+++ b/deepshika.xlsx
@@ -659,6 +659,9 @@
       <c r="L6" t="str">
         <v>Categories page opens successfully in the new tab.</v>
       </c>
+      <c r="N6" t="str">
+        <v>Pass</v>
+      </c>
     </row>
     <row r="7" xml:space="preserve">
       <c r="A7" t="str">
@@ -1542,7 +1545,7 @@
 3. Original category details remain unchanged.</v>
       </c>
       <c r="N25" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R25" t="str">
         <v>Staging</v>
@@ -1903,7 +1906,7 @@
 3. Pagination range/count updates correctly.</v>
       </c>
       <c r="N31" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R31" t="str">
         <v>Staging</v>
@@ -1969,7 +1972,7 @@
 4. Previous/Next controls are enabled or disabled appropriately.</v>
       </c>
       <c r="N32" t="str">
-        <v>Not Tested</v>
+        <v>Pass</v>
       </c>
       <c r="R32" t="str">
         <v>Staging</v>
@@ -2018,6 +2021,9 @@
       <c r="L33" t="str">
         <v>The category associated with the entered slug is displayed and irrelevant categories are excluded.</v>
       </c>
+      <c r="N33" t="str">
+        <v>Pass</v>
+      </c>
     </row>
     <row r="34" xml:space="preserve">
       <c r="A34" t="str">
@@ -2052,6 +2058,9 @@
       <c r="L34" t="str">
         <v>The search criteria is removed and the default category listing is restored.</v>
       </c>
+      <c r="N34" t="str">
+        <v>Pass</v>
+      </c>
     </row>
     <row r="35" xml:space="preserve">
       <c r="A35" t="str">
@@ -2089,6 +2098,9 @@
       </c>
       <c r="L35" t="str">
         <v>The New Category form opens successfully and all expected category input controls are displayed.</v>
+      </c>
+      <c r="N35" t="str">
+        <v>Pass</v>
       </c>
     </row>
     <row r="36">
@@ -2145,6 +2157,9 @@
 6.Table should display maximum 10 records
 7.Table should display maximum 20 records</v>
       </c>
+      <c r="N38" t="str">
+        <v>Pass</v>
+      </c>
     </row>
     <row r="39" xml:space="preserve">
       <c r="A39" t="str">
@@ -2183,6 +2198,9 @@
 4.Pagination controls should be displayed.
 5.User should navigate to the next page
 6.User should return to page 1</v>
+      </c>
+      <c r="N39" t="str">
+        <v>Pass</v>
       </c>
     </row>
   </sheetData>

</xml_diff>